<commit_message>
goods-update.xlsx: Trixie bag barcodes already on unit 001 — move, don't add (checked against the export)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/final/armsoft-2026-10-16/goods-update.xlsx
+++ b/final/armsoft-2026-10-16/goods-update.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'1 RC bags'!$6:$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'2 RC boxes'!$5:$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'3 Felix'!$5:$5</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'4 Weight goods'!$7:$7</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'4 Weight goods'!$9:$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3249,7 +3249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3258,8 +3258,8 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
@@ -3297,194 +3297,100 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
+          <t>Trixie (0403 0459 0516 0517 0552): the bag barcode is ALREADY in ArmSoft, on unit 001: move it to 003, don't add it twice. Only the PLU is new.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Pro Plan 1478 has no barcode at all yet: add both.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
           <t>If ArmSoft refuses to change the main unit (the good already has sales/receipts), tell me and we will find another way.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Name in ArmSoft</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>a) Main unit</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>b) Weight good</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>c) Unit 003 coefficient (bag kg)</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>d) Barcode on 003 (bag)</t>
         </is>
       </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>d) Barcode on 303 = PLU</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>Main barcode</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>e) Price 003 bag (AMD)</t>
         </is>
       </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>e) Price 303 per kg (AMD)</t>
         </is>
       </c>
-      <c r="L7" s="5" t="inlineStr">
+      <c r="L9" s="5" t="inlineStr">
         <is>
           <t>Done ✓</t>
         </is>
       </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>0403</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>Հյուր. շն. Bony Mix` գուն. Ոսկ. կգ</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Trixie Soft Snack Bony Mix XXL / 1,800 g</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>303 (kg)</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>1.8</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>4011905315263</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>00107</t>
-        </is>
-      </c>
-      <c r="I8" s="8" t="inlineStr">
-        <is>
-          <t>00107</t>
-        </is>
-      </c>
-      <c r="J8" s="11" t="n">
-        <v>11500</v>
-      </c>
-      <c r="K8" s="11" t="n">
-        <v>7000</v>
-      </c>
-      <c r="L8" s="7" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>0459</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Պեչենի շն.` գունավոր օղակներ Vegan Loops, կգ</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Trixie Cookie Snack Loops / 1.3 kg</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>303 (kg)</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F9" s="10" t="inlineStr">
-        <is>
-          <t>1.3</t>
-        </is>
-      </c>
-      <c r="G9" s="10" t="inlineStr">
-        <is>
-          <t>4011905316710</t>
-        </is>
-      </c>
-      <c r="H9" s="10" t="inlineStr">
-        <is>
-          <t>00111</t>
-        </is>
-      </c>
-      <c r="I9" s="10" t="inlineStr">
-        <is>
-          <t>00111</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>5980</v>
-      </c>
-      <c r="K9" s="12" t="n">
-        <v>6600</v>
-      </c>
-      <c r="L9" s="9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>0516</t>
+          <t>0403</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>Պեչենի շն.` գունավոր խառը ոսկորիկներ, մեծ կգ</t>
+          <t>Հյուր. շն. Bony Mix` գուն. Ոսկ. կգ</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Trixie Cookie Bones / 1.3 kg</t>
+          <t>Trixie Soft Snack Bony Mix XXL / 1,800 g</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -3499,46 +3405,46 @@
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>4011905316628</t>
+          <t>4011905315263  (already on 001: move it)</t>
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr">
         <is>
-          <t>00108</t>
+          <t>00107  (new)</t>
         </is>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
-          <t>00108</t>
+          <t>00107</t>
         </is>
       </c>
       <c r="J10" s="11" t="n">
-        <v>4900</v>
+        <v>11500</v>
       </c>
       <c r="K10" s="11" t="n">
-        <v>5500</v>
+        <v>7000</v>
       </c>
       <c r="L10" s="7" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>0517</t>
+          <t>0459</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Պեչենի շն.` գունավոր մանր կենդանիներ, Farmies կգ</t>
+          <t>Պեչենի շն.` գունավոր օղակներ Vegan Loops, կգ</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Trixie Cookie Farmies / 1.3 kg</t>
+          <t>Trixie Cookie Snack Loops / 1.3 kg</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
@@ -3558,41 +3464,41 @@
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>4011905316635</t>
+          <t>4011905316710  (already on 001: move it)</t>
         </is>
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>00109</t>
+          <t>00111  (new)</t>
         </is>
       </c>
       <c r="I11" s="10" t="inlineStr">
         <is>
-          <t>00109</t>
+          <t>00111</t>
         </is>
       </c>
       <c r="J11" s="12" t="n">
-        <v>4900</v>
+        <v>5980</v>
       </c>
       <c r="K11" s="12" t="n">
-        <v>5500</v>
+        <v>6600</v>
       </c>
       <c r="L11" s="9" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>0552</t>
+          <t>0516</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>Թխվածքաբլիթներ շն.` գառան մսով, կգ</t>
+          <t>Պեչենի շն.` գունավոր խառը ոսկորիկներ, մեծ կգ</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Trixie Cookie Giants with Lamb / 1.25 kg</t>
+          <t>Trixie Cookie Bones / 1.3 kg</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -3607,85 +3513,193 @@
       </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>1.25</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>4011905316642</t>
+          <t>4011905316628  (already on 001: move it)</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
         <is>
-          <t>00110</t>
+          <t>00108  (new)</t>
         </is>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
-          <t>00110</t>
+          <t>00108</t>
         </is>
       </c>
       <c r="J12" s="11" t="n">
-        <v>4250</v>
+        <v>4900</v>
       </c>
       <c r="K12" s="11" t="n">
-        <v>5700</v>
+        <v>5500</v>
       </c>
       <c r="L12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
+          <t>0517</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Պեչենի շն.` գունավոր մանր կենդանիներ, Farmies կգ</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Trixie Cookie Farmies / 1.3 kg</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>303 (kg)</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>4011905316635  (already on 001: move it)</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>00109  (new)</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>00109</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="n">
+        <v>4900</v>
+      </c>
+      <c r="K13" s="12" t="n">
+        <v>5500</v>
+      </c>
+      <c r="L13" s="9" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>0552</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Թխվածքաբլիթներ շն.` գառան մսով, կգ</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Trixie Cookie Giants with Lamb / 1.25 kg</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>303 (kg)</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>1.25</t>
+        </is>
+      </c>
+      <c r="G14" s="8" t="inlineStr">
+        <is>
+          <t>4011905316642  (already on 001: move it)</t>
+        </is>
+      </c>
+      <c r="H14" s="8" t="inlineStr">
+        <is>
+          <t>00110  (new)</t>
+        </is>
+      </c>
+      <c r="I14" s="8" t="inlineStr">
+        <is>
+          <t>00110</t>
+        </is>
+      </c>
+      <c r="J14" s="11" t="n">
+        <v>4250</v>
+      </c>
+      <c r="K14" s="11" t="n">
+        <v>5700</v>
+      </c>
+      <c r="L14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
           <t>1478</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Pro Plan Cat Sterilised Adult Turkey 10 kg - կատվի կեր 12390976</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>Pro Plan Sterilised Adult Renal Plus / 10 kg</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>303 (kg)</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E15" s="9" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr">
+      <c r="F15" s="10" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="G13" s="10" t="inlineStr">
-        <is>
-          <t>7613033566547</t>
-        </is>
-      </c>
-      <c r="H13" s="10" t="inlineStr">
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>7613033566547  (new)</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>00106  (new)</t>
+        </is>
+      </c>
+      <c r="I15" s="10" t="inlineStr">
         <is>
           <t>00106</t>
         </is>
       </c>
-      <c r="I13" s="10" t="inlineStr">
-        <is>
-          <t>00106</t>
-        </is>
-      </c>
-      <c r="J13" s="12" t="n">
+      <c r="J15" s="12" t="n">
         <v>39500</v>
       </c>
-      <c r="K13" s="12" t="n">
+      <c r="K15" s="12" t="n">
         <v>3950</v>
       </c>
-      <c r="L13" s="9" t="inlineStr"/>
+      <c r="L15" s="9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>